<commit_message>
daily summary: 2026-06-28 (7 videos)
</commit_message>
<xml_diff>
--- a/video_log.xlsx
+++ b/video_log.xlsx
@@ -430,7 +430,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K599"/>
+  <dimension ref="A1:K606"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -39909,6 +39909,479 @@
         </is>
       </c>
     </row>
+    <row r="600">
+      <c r="A600" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-27</t>
+        </is>
+      </c>
+      <c r="B600" s="2" t="inlineStr">
+        <is>
+          <t>タマゴローRS</t>
+        </is>
+      </c>
+      <c r="C600" s="2" t="inlineStr">
+        <is>
+          <t>【ロマサガRS】無尽塔30層「必勝」長期戦!!メタルアルカイザー!!背水無しで精度の高いダメブロ戦立ち回りを構築せよ　#ロマサガRS</t>
+        </is>
+      </c>
+      <c r="D600" s="2" t="inlineStr">
+        <is>
+          <t>無尽塔30層メタルアルカイザーを攻略
+序盤フラワーサンクチュアリでダメブロ安定化
+ビクトル軸＋ネメシス追撃で長期戦を完遂</t>
+        </is>
+      </c>
+      <c r="E600" s="2" t="inlineStr">
+        <is>
+          <t>・背水なしでも精度の高いダメブロ立ち回りで安定
+・終盤は敵攻撃がぬるくなり全力オートでOK
+・携帯タイマーで張り付き不要、ゆっくり攻略可能</t>
+        </is>
+      </c>
+      <c r="F600" s="2" t="inlineStr">
+        <is>
+          <t>・全体範囲攻撃が多いターンは横1列のもらい事故に注意
+・序盤2ターンは敵の全体攻撃が多く不安定</t>
+        </is>
+      </c>
+      <c r="G600" s="2" t="inlineStr">
+        <is>
+          <t>・無尽塔30層
+・メタルアルカイザー
+・ダメブロ構成
+・フラワーサンクチュアリ
+・ビクトル
+・全力オート</t>
+        </is>
+      </c>
+      <c r="H600" s="2" t="inlineStr">
+        <is>
+          <t>ロマサガRS, レイド, ガチャ, 速報</t>
+        </is>
+      </c>
+      <c r="I600" s="2" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=Pj-VU_c5GDU</t>
+        </is>
+      </c>
+      <c r="J600" s="2" t="inlineStr">
+        <is>
+          <t>Pj-VU_c5GDU</t>
+        </is>
+      </c>
+      <c r="K600" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-28T01:05:39Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="601">
+      <c r="A601" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-27</t>
+        </is>
+      </c>
+      <c r="B601" s="2" t="inlineStr">
+        <is>
+          <t>あんずもん</t>
+        </is>
+      </c>
+      <c r="C601" s="2" t="inlineStr">
+        <is>
+          <t>【信長の野望出陣】プレイ開始268日目記録　脅威　果たして２将星は取るべきか？</t>
+        </is>
+      </c>
+      <c r="D601" s="2" t="inlineStr">
+        <is>
+          <t>信長の野望出陣プレイ268日目の進捗報告
+新キャラ10体入手、竜造寺系が大量に集結
+勢力戦・共闘の反省と今後の目標を整理</t>
+        </is>
+      </c>
+      <c r="E601" s="2" t="inlineStr">
+        <is>
+          <t>・別枠イベントがあるのは育成に有効でありがたい
+・長宗我部盛親を1覚醒でき成長を実感
+・立花宗茂は軽減率が高く補填20秒も大きい</t>
+        </is>
+      </c>
+      <c r="F601" s="2" t="inlineStr">
+        <is>
+          <t>・共闘は対応キャラ不足で10位以内が取れない
+・勢力戦は強敵武将の城は取り返され戦力差が無意味
+・オートタイプ不足で小早川を取っても活かしづらい</t>
+        </is>
+      </c>
+      <c r="G601" s="2" t="inlineStr">
+        <is>
+          <t>・信長の野望出陣
+・キャラ入手状況
+・勢力戦
+・共闘
+・開発・神社
+・立花宗茂</t>
+        </is>
+      </c>
+      <c r="H601" s="2" t="inlineStr">
+        <is>
+          <t>ロマサガRS, ライブ配信, コミュニティ</t>
+        </is>
+      </c>
+      <c r="I601" s="2" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=mSnCkoOApCE</t>
+        </is>
+      </c>
+      <c r="J601" s="2" t="inlineStr">
+        <is>
+          <t>mSnCkoOApCE</t>
+        </is>
+      </c>
+      <c r="K601" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-28T01:05:39Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="602">
+      <c r="A602" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-27</t>
+        </is>
+      </c>
+      <c r="B602" s="2" t="inlineStr">
+        <is>
+          <t>つむつむちゃんねる●ゲーム考察専門</t>
+        </is>
+      </c>
+      <c r="C602" s="2" t="inlineStr">
+        <is>
+          <t>【ロマサガRS】総決算7.5周年最強キャラランキング★Tier表更新【ロマンシングサガリユニバース】</t>
+        </is>
+      </c>
+      <c r="D602" s="2" t="inlineStr">
+        <is>
+          <t>7.5周年総決算の最強キャラTier表を更新
+5月実装キャラを卒業させ環境を再整理
+無人島・交代・西王アビリティの環境変化を解説</t>
+        </is>
+      </c>
+      <c r="E602" s="2" t="inlineStr">
+        <is>
+          <t>・西王のアビリティが無人島で刺さり環境支配級
+・ビクトルはEX継承で超級・無人島まで万能で残留
+・検証技なしスタイルを従来以上に高評価</t>
+        </is>
+      </c>
+      <c r="F602" s="2" t="inlineStr">
+        <is>
+          <t>・5月実装のAランク勢は威力不足で軒並み卒業
+・ターミンはパワー不足で環境支配級から陥落
+・無人島は交代でバフ消され火力が出にくい</t>
+        </is>
+      </c>
+      <c r="G602" s="2" t="inlineStr">
+        <is>
+          <t>・7.5周年Tier表
+・卒業式
+・無人島
+・交代(レアス)
+・西王アビス
+・ビクトル</t>
+        </is>
+      </c>
+      <c r="H602" s="2" t="inlineStr">
+        <is>
+          <t>ロマサガRS, 性能考察, ランキング</t>
+        </is>
+      </c>
+      <c r="I602" s="2" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=5kILob7Vz5E</t>
+        </is>
+      </c>
+      <c r="J602" s="2" t="inlineStr">
+        <is>
+          <t>5kILob7Vz5E</t>
+        </is>
+      </c>
+      <c r="K602" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-28T01:05:39Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="603">
+      <c r="A603" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-27</t>
+        </is>
+      </c>
+      <c r="B603" s="2" t="inlineStr">
+        <is>
+          <t>つむつむちゃんねる●ゲーム考察専門</t>
+        </is>
+      </c>
+      <c r="C603" s="2" t="inlineStr">
+        <is>
+          <t>【ロマサガRS】超性能の怪物現る！最新キャラランキング★7.5周年final【ロマンシングサガリユニバース】</t>
+        </is>
+      </c>
+      <c r="D603" s="2" t="inlineStr">
+        <is>
+          <t>7.5周年final最新キャラランキングを発表
+5月実装キャラ卒業＋意外なキャラも整理
+螺旋・討伐・集会・無人島を同列に評価</t>
+        </is>
+      </c>
+      <c r="E603" s="2" t="inlineStr">
+        <is>
+          <t>・検証技なしスタイルは従来以上に評価アップ
+・ビクトルは見切り回避で無人島でも使え残留
+・西王アビリティが環境支配級で刺さる</t>
+        </is>
+      </c>
+      <c r="F603" s="2" t="inlineStr">
+        <is>
+          <t>・無人島が強いだけでは最強とはしない評価基準
+・ターミンはメスのパワー不足で卒業
+・Aランク勢は威力不足で多数卒業</t>
+        </is>
+      </c>
+      <c r="G603" s="2" t="inlineStr">
+        <is>
+          <t>・最新キャラランキング
+・7.5周年final
+・卒業ルール
+・無人島評価
+・ビクトル
+・ターミン</t>
+        </is>
+      </c>
+      <c r="H603" s="2" t="inlineStr">
+        <is>
+          <t>ロマサガRS, 性能考察, ランキング</t>
+        </is>
+      </c>
+      <c r="I603" s="2" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=t0aLk4diRYk</t>
+        </is>
+      </c>
+      <c r="J603" s="2" t="inlineStr">
+        <is>
+          <t>t0aLk4diRYk</t>
+        </is>
+      </c>
+      <c r="K603" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-28T01:05:39Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="604">
+      <c r="A604" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-27</t>
+        </is>
+      </c>
+      <c r="B604" s="2" t="inlineStr">
+        <is>
+          <t>サンゾーGAMES</t>
+        </is>
+      </c>
+      <c r="C604" s="2" t="inlineStr">
+        <is>
+          <t>【ロマサガRS】本当に申し訳ありませんでした！水着ガチャ対決＃3浦田優編【ロマンシング サガ リユニバース】</t>
+        </is>
+      </c>
+      <c r="D604" s="2" t="inlineStr">
+        <is>
+          <t>男3人による水着ガチャ対決の最終戦
+浦田の録画ミスで罰ゲーム(青汁)を実施
+新グループ名「ガムシャラ3」を提案</t>
+        </is>
+      </c>
+      <c r="E604" s="2" t="inlineStr">
+        <is>
+          <t>・70連でコンプした引きを「だいぶ強い」と称賛
+・3人グループ始動で反響が大きく好評</t>
+        </is>
+      </c>
+      <c r="F604" s="2" t="inlineStr">
+        <is>
+          <t>・浦田の画面録画ミスで対決映像が出せず謝罪
+・名前候補は大人の事情で使えないものがある</t>
+        </is>
+      </c>
+      <c r="G604" s="2" t="inlineStr">
+        <is>
+          <t>・水着ガチャ対決
+・ガチャ天井
+・罰ゲーム
+・グループ名
+・ガムシャラ3</t>
+        </is>
+      </c>
+      <c r="H604" s="2" t="inlineStr">
+        <is>
+          <t>ロマサガRS, 攻略全般</t>
+        </is>
+      </c>
+      <c r="I604" s="2" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=ijll8ZM1kWg</t>
+        </is>
+      </c>
+      <c r="J604" s="2" t="inlineStr">
+        <is>
+          <t>ijll8ZM1kWg</t>
+        </is>
+      </c>
+      <c r="K604" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-28T01:05:39Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="605">
+      <c r="A605" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-27</t>
+        </is>
+      </c>
+      <c r="B605" s="2" t="inlineStr">
+        <is>
+          <t>あっきゃんGAMES</t>
+        </is>
+      </c>
+      <c r="C605" s="2" t="inlineStr">
+        <is>
+          <t>【ロマサガRS】7.5周年使い込んだ結論。結局1番の当たりはあのキャラでした【ロマンシングサガリユニバース】</t>
+        </is>
+      </c>
+      <c r="D605" s="2" t="inlineStr">
+        <is>
+          <t>7.5周年実装キャラを使い込んだ最終評価
+裁判・暦み・サライが全コンテンツで活躍
+当たり1位は万能の裁判という結論</t>
+        </is>
+      </c>
+      <c r="E605" s="2" t="inlineStr">
+        <is>
+          <t>・裁判は全コンテンツで活躍する文句なし最高評価
+・暦みは弱点無視の圧倒的火力で周回短縮
+・サライはウィークEXと状態異常解除が優秀
+・ストライフは代償ダメでレイド気絶周回に好相性
+・黒エは意外と火力が出てゴリ押し編成に重宝</t>
+        </is>
+      </c>
+      <c r="F605" s="2" t="inlineStr">
+        <is>
+          <t>・代々はレイド・集会では瞬間火力不足で出番なし
+・黒エは火ダメ軽減率が低く防御面に工夫が必要</t>
+        </is>
+      </c>
+      <c r="G605" s="2" t="inlineStr">
+        <is>
+          <t>・7.5周年キャラ評価
+・裁判
+・暦み
+・サライ
+・ストライフ
+・トップ3</t>
+        </is>
+      </c>
+      <c r="H605" s="2" t="inlineStr">
+        <is>
+          <t>ロマサガRS, 初心者向け, 攻略解説, ショート</t>
+        </is>
+      </c>
+      <c r="I605" s="2" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=jnMdv-T2OBY</t>
+        </is>
+      </c>
+      <c r="J605" s="2" t="inlineStr">
+        <is>
+          <t>jnMdv-T2OBY</t>
+        </is>
+      </c>
+      <c r="K605" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-28T01:05:39Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="606">
+      <c r="A606" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-27</t>
+        </is>
+      </c>
+      <c r="B606" s="2" t="inlineStr">
+        <is>
+          <t>ジュラのサガちゃんねる</t>
+        </is>
+      </c>
+      <c r="C606" s="2" t="inlineStr">
+        <is>
+          <t>【ロマサガRS】高難易度苦手でも29層目指せる「第5回！雲の上の無尽塔」【ロマンシング サガ リユニバース】</t>
+        </is>
+      </c>
+      <c r="D606" s="2" t="inlineStr">
+        <is>
+          <t>無人島(無尽塔)29層までの攻略ワンポイント解説
+7層ペンギン・15層守護者・20層バウムが関門
+30層メタルアルカイザーは別格で対象外</t>
+        </is>
+      </c>
+      <c r="E606" s="2" t="inlineStr">
+        <is>
+          <t>・7.5周年キャラがあれば26層まで全力オート可能
+・各階突破でジュエルが貰えてお得
+・ポルカ・オタマはセレチケ交換でダメブロ要員に</t>
+        </is>
+      </c>
+      <c r="F606" s="2" t="inlineStr">
+        <is>
+          <t>・30層メタルアルカイザーは意味不明な難易度で対象外
+・無人島は大味すぎて別の味変コンテンツが欲しい
+・15層守護者・20層バウムはギミック知らないと苦戦</t>
+        </is>
+      </c>
+      <c r="G606" s="2" t="inlineStr">
+        <is>
+          <t>・雲の上の無人島
+・29層攻略
+・皇帝ペンギン
+・守護者ギミック
+・ゴールデンバウム
+・ダメブロ</t>
+        </is>
+      </c>
+      <c r="H606" s="2" t="inlineStr">
+        <is>
+          <t>ロマサガRS, ガチャ, ランキング</t>
+        </is>
+      </c>
+      <c r="I606" s="2" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=h9ZuPjaeq5s</t>
+        </is>
+      </c>
+      <c r="J606" s="2" t="inlineStr">
+        <is>
+          <t>h9ZuPjaeq5s</t>
+        </is>
+      </c>
+      <c r="K606" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-28T01:05:39Z</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:K1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>